<commit_message>
Archivos de imagenes y demas
</commit_message>
<xml_diff>
--- a/Data/Procesados/Resultados_Congruencia_General.xlsx
+++ b/Data/Procesados/Resultados_Congruencia_General.xlsx
@@ -485,16 +485,16 @@
         <v>2786</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7968413496051687</v>
+        <v>0.1138344785150241</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.717516152189519</v>
+        <v>-0.1025023074556456</v>
       </c>
       <c r="F2" t="n">
-        <v>651078.5</v>
+        <v>651770.5</v>
       </c>
       <c r="G2" t="n">
-        <v>3.110308076721872e-41</v>
+        <v>5.960375019981098e-41</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -517,16 +517,16 @@
         <v>2786</v>
       </c>
       <c r="D3" t="n">
-        <v>-20.18418395549174</v>
+        <v>-2.883454850784535</v>
       </c>
       <c r="E3" t="n">
-        <v>-18.7597916367552</v>
+        <v>-2.679970233822172</v>
       </c>
       <c r="F3" t="n">
-        <v>1568324.5</v>
+        <v>1568319.5</v>
       </c>
       <c r="G3" t="n">
-        <v>2.094839874154954e-18</v>
+        <v>2.092653477752801e-18</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -549,16 +549,16 @@
         <v>1254</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3373205741626794</v>
+        <v>0.04818865345181136</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.2240829346092504</v>
+        <v>-0.03201184780132148</v>
       </c>
       <c r="F4" t="n">
-        <v>168625</v>
+        <v>168319</v>
       </c>
       <c r="G4" t="n">
-        <v>0.009005260591428492</v>
+        <v>0.008078134899648662</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -581,16 +581,16 @@
         <v>1254</v>
       </c>
       <c r="D5" t="n">
-        <v>-18.37136483253589</v>
+        <v>-2.624480690362269</v>
       </c>
       <c r="E5" t="n">
-        <v>-16.82836403508772</v>
+        <v>-2.404052005012531</v>
       </c>
       <c r="F5" t="n">
-        <v>335299.5</v>
+        <v>335300.5</v>
       </c>
       <c r="G5" t="n">
-        <v>5.8162230014155e-06</v>
+        <v>5.81837095387041e-06</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>

</xml_diff>